<commit_message>
① 取值约束：min / max / choices / pattern
工具此前只查"变量有没有定义、类型对不对"，完全不看值 —— 把 20.559 手滑打成
205.59 会一路渲染成错误代码，而 check 只会说"与参数一致"。这是唯一一类
"工具不报错但交付物是错的"的缺口。

- VariableDef 新增 min / max / choices / pattern；配置期拦住写错的约束
  （min>max、给 string 加范围、default 越界、派生参数加约束、坏的正则……）
- 新增 check_value_constraints()：render / validate -x / check 每次读表后校验，
  一次列出全部问题并指出表、列、Case、变量；越界退出码 1
- create_template 把约束写成 Excel 数据有效性：choices → 下拉列表，
  min/max → 整数/小数范围，带悬停提示；判据仍是工具侧那道闸
- 空值算不合格 —— 顺手治了"新插空 Case 列悄悄落进某个规则集"的老问题
- 表达不了就报错：下拉选项含逗号或超 255 字符 → 报错；pattern 不写数据有效性
- examples/example.yaml 加上约束示例；指南新增 §3.5；cli.md / README 同步

测试：新增 tests/test_constraints.py 29 项，全量 136 项通过；
abs_fpi/build.py --check 公式求值 28 项 0 失败。
</commit_message>
<xml_diff>
--- a/examples/template.xlsx
+++ b/examples/template.xlsx
@@ -655,7 +655,7 @@
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  时间        2026-09-24 16:59:16</t>
+          <t xml:space="preserve">  时间        2026-09-27 13:10:03</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  命令      excel-codegen render -c examples\example.yaml -x examples\template.xlsx --write-excel --outdir examples\generated</t>
+          <t xml:space="preserve">  命令      excel-codegen render -c examples/example.yaml -x examples/template.xlsx --write-excel --outdir examples/generated</t>
         </is>
       </c>
     </row>
@@ -808,6 +808,12 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="取值不合规" error="baud：范围: 300 ~ 4000000" promptTitle="baud" prompt="范围: 300 ~ 4000000" type="whole" operator="between">
+      <formula1>300</formula1>
+      <formula2>4000000</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -901,7 +907,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>模式</t>
+          <t>模式（取值约束：Excel 里会变成下拉列表）</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -921,6 +927,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E3 F3" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="取值不合规" error="mode：可选: TX / RX / TX_RX" promptTitle="mode" prompt="可选: TX / RX / TX_RX" type="list">
+      <formula1>"TX,RX,TX_RX"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1413,7 +1424,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-24 16:59:16</t>
+          <t>2026-09-27 13:10:03</t>
         </is>
       </c>
     </row>

</xml_diff>